<commit_message>
feat: add project intake template, highlight mandatory/optional fields, enable AI auto-generation and project editing
- Remove demo references from UI copy to make application enterprise deployment ready
- Generate minimal project intake template (10 fields max) with mandatory vs optional fields visually highlighted
- Highlight mandatory and optional headers across all portfolio Excel files in data/portfolios
- Support AI auto-generation of remaining PMO signals, scores, rules, and drivers on template import
- Build Edit Project screen and modal allowing users to inspect and adjust all core and AI-generated fields

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/portfolios/portfolio_ai_team.xlsx
+++ b/data/portfolios/portfolio_ai_team.xlsx
@@ -36,7 +36,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -45,8 +45,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000078D4"/>
-        <bgColor rgb="000078D4"/>
+        <fgColor rgb="00004578"/>
+        <bgColor rgb="00004578"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="005C6873"/>
+        <bgColor rgb="005C6873"/>
       </patternFill>
     </fill>
   </fills>
@@ -76,10 +82,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -453,1651 +462,1651 @@
   <dimension ref="A1:AI11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="54" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="17" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="23" customWidth="1" min="12" max="12"/>
-    <col width="24" customWidth="1" min="13" max="13"/>
-    <col width="25" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
-    <col width="27" customWidth="1" min="16" max="16"/>
-    <col width="21" customWidth="1" min="17" max="17"/>
-    <col width="22" customWidth="1" min="18" max="18"/>
-    <col width="19" customWidth="1" min="19" max="19"/>
-    <col width="14" customWidth="1" min="20" max="20"/>
-    <col width="24" customWidth="1" min="21" max="21"/>
-    <col width="15" customWidth="1" min="22" max="22"/>
-    <col width="12" customWidth="1" min="23" max="23"/>
-    <col width="18" customWidth="1" min="24" max="24"/>
-    <col width="19" customWidth="1" min="25" max="25"/>
-    <col width="19" customWidth="1" min="26" max="26"/>
+    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="29" customWidth="1" min="6" max="6"/>
+    <col width="31" customWidth="1" min="7" max="7"/>
+    <col width="27" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="31" customWidth="1" min="11" max="11"/>
+    <col width="37" customWidth="1" min="12" max="12"/>
+    <col width="35" customWidth="1" min="13" max="13"/>
+    <col width="36" customWidth="1" min="14" max="14"/>
+    <col width="31" customWidth="1" min="15" max="15"/>
+    <col width="30" customWidth="1" min="16" max="16"/>
+    <col width="32" customWidth="1" min="17" max="17"/>
+    <col width="36" customWidth="1" min="18" max="18"/>
+    <col width="30" customWidth="1" min="19" max="19"/>
+    <col width="25" customWidth="1" min="20" max="20"/>
+    <col width="35" customWidth="1" min="21" max="21"/>
+    <col width="26" customWidth="1" min="22" max="22"/>
+    <col width="21" customWidth="1" min="23" max="23"/>
+    <col width="29" customWidth="1" min="24" max="24"/>
+    <col width="30" customWidth="1" min="25" max="25"/>
+    <col width="30" customWidth="1" min="26" max="26"/>
     <col width="28" customWidth="1" min="27" max="27"/>
     <col width="28" customWidth="1" min="28" max="28"/>
-    <col width="17" customWidth="1" min="29" max="29"/>
-    <col width="25" customWidth="1" min="30" max="30"/>
-    <col width="12" customWidth="1" min="31" max="31"/>
-    <col width="56" customWidth="1" min="32" max="32"/>
-    <col width="104" customWidth="1" min="33" max="33"/>
-    <col width="45" customWidth="1" min="34" max="34"/>
-    <col width="18" customWidth="1" min="35" max="35"/>
+    <col width="28" customWidth="1" min="29" max="29"/>
+    <col width="32" customWidth="1" min="30" max="30"/>
+    <col width="21" customWidth="1" min="31" max="31"/>
+    <col width="40" customWidth="1" min="32" max="32"/>
+    <col width="40" customWidth="1" min="33" max="33"/>
+    <col width="40" customWidth="1" min="34" max="34"/>
+    <col width="29" customWidth="1" min="35" max="35"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Project ID</t>
+          <t>Project ID * [MANDATORY]</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Project Name</t>
+          <t>Project Name * [MANDATORY]</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Portfolio</t>
+          <t>Portfolio * [MANDATORY]</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Business Unit</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Site</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Project Manager</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Executive Sponsor</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Sponsor Level</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Project Status</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Go-Live Date</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Months to Go-Live</t>
+          <t>Business Unit * [MANDATORY]</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Site [OPTIONAL]</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Project Manager [OPTIONAL]</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Executive Sponsor [OPTIONAL]</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Sponsor Level [OPTIONAL]</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Project Status [OPTIONAL]</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Go-Live Date [OPTIONAL]</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Months to Go-Live [OPTIONAL]</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Business Value (1-5)</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Regulatory / Security</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Digital Transformation</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Protected Program</t>
+          <t>Business Value (1-5) * [MANDATORY]</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Regulatory / Security [OPTIONAL]</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>Digital Transformation [OPTIONAL]</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>Protected Program [OPTIONAL]</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>Primary Skill</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Skill Demand (FTE)</t>
+          <t>Primary Skill * [MANDATORY]</t>
+        </is>
+      </c>
+      <c r="Q1" s="2" t="inlineStr">
+        <is>
+          <t>Skill Demand (FTE) [OPTIONAL]</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>Cost Estimate (USD)</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>Dependency Count</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>Risk Rating</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>Effort (Person-Weeks)</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>Completeness</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>Quality</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>Model Certainty</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>Confidence Score</t>
-        </is>
-      </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>Confidence Level</t>
-        </is>
-      </c>
-      <c r="AA1" s="1" t="inlineStr">
-        <is>
-          <t>ML Tier</t>
-        </is>
-      </c>
-      <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>Final Tier</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>Priority Score</t>
-        </is>
-      </c>
-      <c r="AD1" s="1" t="inlineStr">
-        <is>
-          <t>Recommended Action</t>
-        </is>
-      </c>
-      <c r="AE1" s="1" t="inlineStr">
-        <is>
-          <t>Cluster</t>
-        </is>
-      </c>
-      <c r="AF1" s="1" t="inlineStr">
-        <is>
-          <t>Rule Overrides</t>
-        </is>
-      </c>
-      <c r="AG1" s="1" t="inlineStr">
-        <is>
-          <t>Top Drivers</t>
-        </is>
-      </c>
-      <c r="AH1" s="1" t="inlineStr">
-        <is>
-          <t>Data Issues</t>
-        </is>
-      </c>
-      <c r="AI1" s="1" t="inlineStr">
-        <is>
-          <t>Sources Present</t>
+          <t>Cost Estimate (USD) * [MANDATORY]</t>
+        </is>
+      </c>
+      <c r="S1" s="2" t="inlineStr">
+        <is>
+          <t>Dependency Count [OPTIONAL]</t>
+        </is>
+      </c>
+      <c r="T1" s="2" t="inlineStr">
+        <is>
+          <t>Risk Rating [OPTIONAL]</t>
+        </is>
+      </c>
+      <c r="U1" s="2" t="inlineStr">
+        <is>
+          <t>Effort (Person-Weeks) [OPTIONAL]</t>
+        </is>
+      </c>
+      <c r="V1" s="2" t="inlineStr">
+        <is>
+          <t>Completeness [OPTIONAL]</t>
+        </is>
+      </c>
+      <c r="W1" s="2" t="inlineStr">
+        <is>
+          <t>Quality [OPTIONAL]</t>
+        </is>
+      </c>
+      <c r="X1" s="2" t="inlineStr">
+        <is>
+          <t>Model Certainty [OPTIONAL]</t>
+        </is>
+      </c>
+      <c r="Y1" s="2" t="inlineStr">
+        <is>
+          <t>Confidence Score [OPTIONAL]</t>
+        </is>
+      </c>
+      <c r="Z1" s="2" t="inlineStr">
+        <is>
+          <t>Confidence Level [OPTIONAL]</t>
+        </is>
+      </c>
+      <c r="AA1" s="2" t="inlineStr">
+        <is>
+          <t>ML Tier [OPTIONAL]</t>
+        </is>
+      </c>
+      <c r="AB1" s="2" t="inlineStr">
+        <is>
+          <t>Final Tier [OPTIONAL]</t>
+        </is>
+      </c>
+      <c r="AC1" s="2" t="inlineStr">
+        <is>
+          <t>Priority Score [OPTIONAL]</t>
+        </is>
+      </c>
+      <c r="AD1" s="2" t="inlineStr">
+        <is>
+          <t>Recommended Action [OPTIONAL]</t>
+        </is>
+      </c>
+      <c r="AE1" s="2" t="inlineStr">
+        <is>
+          <t>Cluster [OPTIONAL]</t>
+        </is>
+      </c>
+      <c r="AF1" s="2" t="inlineStr">
+        <is>
+          <t>Rule Overrides [OPTIONAL]</t>
+        </is>
+      </c>
+      <c r="AG1" s="2" t="inlineStr">
+        <is>
+          <t>Top Drivers [OPTIONAL]</t>
+        </is>
+      </c>
+      <c r="AH1" s="2" t="inlineStr">
+        <is>
+          <t>Data Issues [OPTIONAL]</t>
+        </is>
+      </c>
+      <c r="AI1" s="2" t="inlineStr">
+        <is>
+          <t>Sources Present [OPTIONAL]</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>GIS-0076</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Wafer Defect Computer Vision Inspection AI</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>AI Team</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>Information Security</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>Tualatin</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>Elena Novak</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Leila Iyer</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>Manager</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>2027-12-15</t>
         </is>
       </c>
-      <c r="K2" s="3" t="n">
+      <c r="K2" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="L2" s="3" t="n">
+      <c r="L2" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="M2" s="3" t="b">
+      <c r="M2" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="N2" s="3" t="b">
+      <c r="N2" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="O2" s="3" t="b">
+      <c r="O2" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="P2" s="2" t="inlineStr">
+      <c r="P2" s="3" t="inlineStr">
         <is>
           <t>Integration (iPaaS)</t>
         </is>
       </c>
-      <c r="Q2" s="3" t="n">
+      <c r="Q2" s="4" t="n">
         <v>6.3</v>
       </c>
-      <c r="R2" s="3" t="n">
+      <c r="R2" s="4" t="n">
         <v>685316</v>
       </c>
-      <c r="S2" s="3" t="n">
+      <c r="S2" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="T2" s="2" t="inlineStr">
+      <c r="T2" s="3" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="U2" s="3" t="n">
+      <c r="U2" s="4" t="n">
         <v>144</v>
       </c>
-      <c r="V2" s="3" t="n">
+      <c r="V2" s="4" t="n">
         <v>0.85</v>
       </c>
-      <c r="W2" s="3" t="n">
+      <c r="W2" s="4" t="n">
         <v>0.84</v>
       </c>
-      <c r="X2" s="3" t="n">
+      <c r="X2" s="4" t="n">
         <v>0.83</v>
       </c>
-      <c r="Y2" s="3" t="n">
+      <c r="Y2" s="4" t="n">
         <v>84.2</v>
       </c>
-      <c r="Z2" s="2" t="inlineStr">
+      <c r="Z2" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="AA2" s="2" t="inlineStr">
+      <c r="AA2" s="3" t="inlineStr">
         <is>
           <t>Must-do-now</t>
         </is>
       </c>
-      <c r="AB2" s="2" t="inlineStr">
+      <c r="AB2" s="3" t="inlineStr">
         <is>
           <t>Must-do-now</t>
         </is>
       </c>
-      <c r="AC2" s="3" t="n">
+      <c r="AC2" s="4" t="n">
         <v>98.5</v>
       </c>
-      <c r="AD2" s="2" t="inlineStr">
+      <c r="AD2" s="3" t="inlineStr">
         <is>
           <t>Protect slot</t>
         </is>
       </c>
-      <c r="AE2" s="2" t="inlineStr">
+      <c r="AE2" s="3" t="inlineStr">
         <is>
           <t>Analytics</t>
         </is>
       </c>
-      <c r="AF2" s="2" t="inlineStr">
+      <c r="AF2" s="3" t="inlineStr">
         <is>
           <t>R3 Protected Program</t>
         </is>
       </c>
-      <c r="AG2" s="2" t="inlineStr">
+      <c r="AG2" s="3" t="inlineStr">
         <is>
           <t>Business Value (+0.90); Timing Urgency (+0.26); Regulatory / Security (-0.12); Cost Magnitude (-0.03)</t>
         </is>
       </c>
-      <c r="AH2" s="2" t="inlineStr"/>
-      <c r="AI2" s="3" t="n">
+      <c r="AH2" s="3" t="inlineStr"/>
+      <c r="AI2" s="4" t="n">
         <v>9</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>GIS-0077</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Generative AI Knowledge Assistant for Fab Engineers</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>AI Team</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Digital Transformation</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>Fremont</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>Jordan Aziz</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Ingrid Iyer</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>Director</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Planning</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>2026-08-09</t>
         </is>
       </c>
-      <c r="K3" s="3" t="n">
+      <c r="K3" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="L3" s="3" t="n">
+      <c r="L3" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="M3" s="3" t="b">
+      <c r="M3" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="N3" s="3" t="b">
+      <c r="N3" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="O3" s="3" t="b">
+      <c r="O3" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="P3" s="2" t="inlineStr">
+      <c r="P3" s="3" t="inlineStr">
         <is>
           <t>Cloud and Infrastructure</t>
         </is>
       </c>
-      <c r="Q3" s="3" t="n">
+      <c r="Q3" s="4" t="n">
         <v>4.8</v>
       </c>
-      <c r="R3" s="3" t="n">
+      <c r="R3" s="4" t="n">
         <v>2238353</v>
       </c>
-      <c r="S3" s="3" t="n">
+      <c r="S3" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="T3" s="2" t="inlineStr">
+      <c r="T3" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="U3" s="3" t="n">
+      <c r="U3" s="4" t="n">
         <v>69</v>
       </c>
-      <c r="V3" s="3" t="n">
+      <c r="V3" s="4" t="n">
         <v>0.83</v>
       </c>
-      <c r="W3" s="3" t="n">
+      <c r="W3" s="4" t="n">
         <v>0.89</v>
       </c>
-      <c r="X3" s="3" t="n">
+      <c r="X3" s="4" t="n">
         <v>0.87</v>
       </c>
-      <c r="Y3" s="3" t="n">
+      <c r="Y3" s="4" t="n">
         <v>85.90000000000001</v>
       </c>
-      <c r="Z3" s="2" t="inlineStr">
+      <c r="Z3" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="AA3" s="2" t="inlineStr">
+      <c r="AA3" s="3" t="inlineStr">
         <is>
           <t>Must-do-now</t>
         </is>
       </c>
-      <c r="AB3" s="2" t="inlineStr">
+      <c r="AB3" s="3" t="inlineStr">
         <is>
           <t>Must-do-now</t>
         </is>
       </c>
-      <c r="AC3" s="3" t="n">
+      <c r="AC3" s="4" t="n">
         <v>78.90000000000001</v>
       </c>
-      <c r="AD3" s="2" t="inlineStr">
+      <c r="AD3" s="3" t="inlineStr">
         <is>
           <t>Proceed</t>
         </is>
       </c>
-      <c r="AE3" s="2" t="inlineStr">
+      <c r="AE3" s="3" t="inlineStr">
         <is>
           <t>Analytics</t>
         </is>
       </c>
-      <c r="AF3" s="2" t="inlineStr">
+      <c r="AF3" s="3" t="inlineStr">
         <is>
           <t>R1 Regulatory First</t>
         </is>
       </c>
-      <c r="AG3" s="2" t="inlineStr">
+      <c r="AG3" s="3" t="inlineStr">
         <is>
           <t>Business Value (+0.36); Timing Urgency (+0.58); Regulatory / Security (+0.45); Cost Magnitude (-0.11)</t>
         </is>
       </c>
-      <c r="AH3" s="2" t="inlineStr"/>
-      <c r="AI3" s="3" t="n">
+      <c r="AH3" s="3" t="inlineStr"/>
+      <c r="AI3" s="4" t="n">
         <v>9</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>GIS-0078</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Predictive Equipment Maintenance Anomaly Detector</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>AI Team</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Customer Services</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Global Remote</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Sophia Patel</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Samuel Lindqvist</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Manager</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Planning</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="K4" s="3" t="n">
+      <c r="K4" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="L4" s="3" t="n">
+      <c r="L4" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="M4" s="3" t="b">
+      <c r="M4" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="N4" s="3" t="b">
+      <c r="N4" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="O4" s="3" t="b">
+      <c r="O4" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="P4" s="2" t="inlineStr">
+      <c r="P4" s="3" t="inlineStr">
         <is>
           <t>Project Management</t>
         </is>
       </c>
-      <c r="Q4" s="3" t="n">
+      <c r="Q4" s="4" t="n">
         <v>2.8</v>
       </c>
-      <c r="R4" s="3" t="n">
+      <c r="R4" s="4" t="n">
         <v>2400000</v>
       </c>
-      <c r="S4" s="3" t="n">
+      <c r="S4" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="T4" s="2" t="inlineStr">
+      <c r="T4" s="3" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="U4" s="3" t="n">
+      <c r="U4" s="4" t="n">
         <v>209</v>
       </c>
-      <c r="V4" s="3" t="n">
+      <c r="V4" s="4" t="n">
         <v>0.64</v>
       </c>
-      <c r="W4" s="3" t="n">
+      <c r="W4" s="4" t="n">
         <v>0.95</v>
       </c>
-      <c r="X4" s="3" t="n">
+      <c r="X4" s="4" t="n">
         <v>0.9</v>
       </c>
-      <c r="Y4" s="3" t="n">
+      <c r="Y4" s="4" t="n">
         <v>80.09999999999999</v>
       </c>
-      <c r="Z4" s="2" t="inlineStr">
+      <c r="Z4" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="AA4" s="2" t="inlineStr">
+      <c r="AA4" s="3" t="inlineStr">
         <is>
           <t>Must-do-now</t>
         </is>
       </c>
-      <c r="AB4" s="2" t="inlineStr">
+      <c r="AB4" s="3" t="inlineStr">
         <is>
           <t>Must-do-now</t>
         </is>
       </c>
-      <c r="AC4" s="3" t="n">
+      <c r="AC4" s="4" t="n">
         <v>98.5</v>
       </c>
-      <c r="AD4" s="2" t="inlineStr">
+      <c r="AD4" s="3" t="inlineStr">
         <is>
           <t>Protect slot</t>
         </is>
       </c>
-      <c r="AE4" s="2" t="inlineStr">
+      <c r="AE4" s="3" t="inlineStr">
         <is>
           <t>Core IT</t>
         </is>
       </c>
-      <c r="AF4" s="2" t="inlineStr">
+      <c r="AF4" s="3" t="inlineStr">
         <is>
           <t>R1 Regulatory First; R3 Protected Program</t>
         </is>
       </c>
-      <c r="AG4" s="2" t="inlineStr">
+      <c r="AG4" s="3" t="inlineStr">
         <is>
           <t>Business Value (+0.72); Timing Urgency (+0.54); Regulatory / Security (+0.45); Cost Magnitude (-0.12)</t>
         </is>
       </c>
-      <c r="AH4" s="2" t="inlineStr"/>
-      <c r="AI4" s="3" t="n">
+      <c r="AH4" s="3" t="inlineStr"/>
+      <c r="AI4" s="4" t="n">
         <v>7</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>GIS-0079</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Supply Chain Disruption Forecasting Model</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>AI Team</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>Fab Operations</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>Tualatin</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>Marcus Aziz</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>Lucas Schmidt</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>Director</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>Planning</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>2028-11-06</t>
         </is>
       </c>
-      <c r="K5" s="3" t="n">
+      <c r="K5" s="4" t="n">
         <v>34</v>
       </c>
-      <c r="L5" s="3" t="n">
+      <c r="L5" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="M5" s="3" t="b">
+      <c r="M5" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="N5" s="3" t="b">
+      <c r="N5" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="O5" s="3" t="b">
+      <c r="O5" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="P5" s="2" t="inlineStr">
+      <c r="P5" s="3" t="inlineStr">
         <is>
           <t>Cloud and Infrastructure</t>
         </is>
       </c>
-      <c r="Q5" s="3" t="n">
+      <c r="Q5" s="4" t="n">
         <v>4.1</v>
       </c>
-      <c r="R5" s="3" t="n">
+      <c r="R5" s="4" t="n">
         <v>1502826</v>
       </c>
-      <c r="S5" s="3" t="n">
+      <c r="S5" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="T5" s="2" t="inlineStr">
+      <c r="T5" s="3" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="U5" s="3" t="n">
+      <c r="U5" s="4" t="n">
         <v>109</v>
       </c>
-      <c r="V5" s="3" t="n">
+      <c r="V5" s="4" t="n">
         <v>0.51</v>
       </c>
-      <c r="W5" s="3" t="n">
+      <c r="W5" s="4" t="n">
         <v>0.75</v>
       </c>
-      <c r="X5" s="3" t="n">
+      <c r="X5" s="4" t="n">
         <v>0.73</v>
       </c>
-      <c r="Y5" s="3" t="n">
+      <c r="Y5" s="4" t="n">
         <v>63.8</v>
       </c>
-      <c r="Z5" s="2" t="inlineStr">
+      <c r="Z5" s="3" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="AA5" s="2" t="inlineStr">
+      <c r="AA5" s="3" t="inlineStr">
         <is>
           <t>Proceed</t>
         </is>
       </c>
-      <c r="AB5" s="2" t="inlineStr">
+      <c r="AB5" s="3" t="inlineStr">
         <is>
           <t>Proceed</t>
         </is>
       </c>
-      <c r="AC5" s="3" t="n">
+      <c r="AC5" s="4" t="n">
         <v>67.59999999999999</v>
       </c>
-      <c r="AD5" s="2" t="inlineStr">
+      <c r="AD5" s="3" t="inlineStr">
         <is>
           <t>Proceed</t>
         </is>
       </c>
-      <c r="AE5" s="2" t="inlineStr">
+      <c r="AE5" s="3" t="inlineStr">
         <is>
           <t>Analytics</t>
         </is>
       </c>
-      <c r="AF5" s="2" t="inlineStr"/>
-      <c r="AG5" s="2" t="inlineStr">
+      <c r="AF5" s="3" t="inlineStr"/>
+      <c r="AG5" s="3" t="inlineStr">
         <is>
           <t>Business Value (+0.72); Timing Urgency (+0.04); Regulatory / Security (-0.12); Cost Magnitude (-0.08)</t>
         </is>
       </c>
-      <c r="AH5" s="2" t="inlineStr">
+      <c r="AH5" s="3" t="inlineStr">
         <is>
           <t>Sparse cross-system presence (&lt; 7 sources)</t>
         </is>
       </c>
-      <c r="AI5" s="3" t="n">
+      <c r="AI5" s="4" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>GIS-0080</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>Automated Recipe Optimization Deep Learning</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>AI Team</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Corporate IT</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>Singapore</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Kenji Kim</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>Sofia Schmidt</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>Executive</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="J6" s="3" t="inlineStr">
         <is>
           <t>2028-02-07</t>
         </is>
       </c>
-      <c r="K6" s="3" t="n">
+      <c r="K6" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="L6" s="3" t="n">
+      <c r="L6" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="M6" s="3" t="b">
+      <c r="M6" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="N6" s="3" t="b">
+      <c r="N6" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="O6" s="3" t="b">
+      <c r="O6" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="P6" s="2" t="inlineStr">
+      <c r="P6" s="3" t="inlineStr">
         <is>
           <t>Application Development</t>
         </is>
       </c>
-      <c r="Q6" s="3" t="n">
+      <c r="Q6" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="R6" s="3" t="n">
+      <c r="R6" s="4" t="n">
         <v>1349076</v>
       </c>
-      <c r="S6" s="3" t="n">
+      <c r="S6" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="T6" s="2" t="inlineStr">
+      <c r="T6" s="3" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="U6" s="3" t="n">
+      <c r="U6" s="4" t="n">
         <v>144</v>
       </c>
-      <c r="V6" s="3" t="n">
+      <c r="V6" s="4" t="n">
         <v>0.61</v>
       </c>
-      <c r="W6" s="3" t="n">
+      <c r="W6" s="4" t="n">
         <v>0.87</v>
       </c>
-      <c r="X6" s="3" t="n">
+      <c r="X6" s="4" t="n">
         <v>0.72</v>
       </c>
-      <c r="Y6" s="3" t="n">
+      <c r="Y6" s="4" t="n">
         <v>72.3</v>
       </c>
-      <c r="Z6" s="2" t="inlineStr">
+      <c r="Z6" s="3" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="AA6" s="2" t="inlineStr">
+      <c r="AA6" s="3" t="inlineStr">
         <is>
           <t>Candidate to deprioritize</t>
         </is>
       </c>
-      <c r="AB6" s="2" t="inlineStr">
+      <c r="AB6" s="3" t="inlineStr">
         <is>
           <t>Candidate to deprioritize</t>
         </is>
       </c>
-      <c r="AC6" s="3" t="n">
+      <c r="AC6" s="4" t="n">
         <v>21.8</v>
       </c>
-      <c r="AD6" s="2" t="inlineStr">
+      <c r="AD6" s="3" t="inlineStr">
         <is>
           <t>Pause or divert skills</t>
         </is>
       </c>
-      <c r="AE6" s="2" t="inlineStr">
+      <c r="AE6" s="3" t="inlineStr">
         <is>
           <t>Core IT</t>
         </is>
       </c>
-      <c r="AF6" s="2" t="inlineStr">
+      <c r="AF6" s="3" t="inlineStr">
         <is>
           <t>R2 Executive Sponsorship</t>
         </is>
       </c>
-      <c r="AG6" s="2" t="inlineStr">
+      <c r="AG6" s="3" t="inlineStr">
         <is>
           <t>Business Value (+0.18); Timing Urgency (+0.22); Regulatory / Security (-0.12); Cost Magnitude (-0.07)</t>
         </is>
       </c>
-      <c r="AH6" s="2" t="inlineStr"/>
-      <c r="AI6" s="3" t="n">
+      <c r="AH6" s="3" t="inlineStr"/>
+      <c r="AI6" s="4" t="n">
         <v>7</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>GIS-0081</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Enterprise LLM Model Serving Gateway</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>AI Team</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>Global Supply Chain</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>Tualatin</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>Isabel Brandt</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>Priya Reyes</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>Manager</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="J7" s="3" t="inlineStr">
         <is>
           <t>2027-09-19</t>
         </is>
       </c>
-      <c r="K7" s="3" t="n">
+      <c r="K7" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="L7" s="3" t="n">
+      <c r="L7" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="M7" s="3" t="b">
+      <c r="M7" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="N7" s="3" t="b">
+      <c r="N7" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="O7" s="3" t="b">
+      <c r="O7" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="P7" s="2" t="inlineStr">
+      <c r="P7" s="3" t="inlineStr">
         <is>
           <t>Data Engineering</t>
         </is>
       </c>
-      <c r="Q7" s="3" t="n">
+      <c r="Q7" s="4" t="n">
         <v>5.2</v>
       </c>
-      <c r="R7" s="3" t="n">
+      <c r="R7" s="4" t="n">
         <v>4800000</v>
       </c>
-      <c r="S7" s="3" t="n">
+      <c r="S7" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="T7" s="2" t="inlineStr">
+      <c r="T7" s="3" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="U7" s="3" t="n">
+      <c r="U7" s="4" t="n">
         <v>65</v>
       </c>
-      <c r="V7" s="3" t="n">
+      <c r="V7" s="4" t="n">
         <v>0.43</v>
       </c>
-      <c r="W7" s="3" t="n">
+      <c r="W7" s="4" t="n">
         <v>0.85</v>
       </c>
-      <c r="X7" s="3" t="n">
+      <c r="X7" s="4" t="n">
         <v>0.83</v>
       </c>
-      <c r="Y7" s="3" t="n">
+      <c r="Y7" s="4" t="n">
         <v>65.7</v>
       </c>
-      <c r="Z7" s="2" t="inlineStr">
+      <c r="Z7" s="3" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="AA7" s="2" t="inlineStr">
+      <c r="AA7" s="3" t="inlineStr">
         <is>
           <t>Proceed</t>
         </is>
       </c>
-      <c r="AB7" s="2" t="inlineStr">
+      <c r="AB7" s="3" t="inlineStr">
         <is>
           <t>Proceed</t>
         </is>
       </c>
-      <c r="AC7" s="3" t="n">
+      <c r="AC7" s="4" t="n">
         <v>68.09999999999999</v>
       </c>
-      <c r="AD7" s="2" t="inlineStr">
+      <c r="AD7" s="3" t="inlineStr">
         <is>
           <t>Proceed</t>
         </is>
       </c>
-      <c r="AE7" s="2" t="inlineStr">
+      <c r="AE7" s="3" t="inlineStr">
         <is>
           <t>Analytics</t>
         </is>
       </c>
-      <c r="AF7" s="2" t="inlineStr"/>
-      <c r="AG7" s="2" t="inlineStr">
+      <c r="AF7" s="3" t="inlineStr"/>
+      <c r="AG7" s="3" t="inlineStr">
         <is>
           <t>Business Value (+0.54); Timing Urgency (+0.32); Regulatory / Security (-0.12); Cost Magnitude (-0.24)</t>
         </is>
       </c>
-      <c r="AH7" s="2" t="inlineStr">
+      <c r="AH7" s="3" t="inlineStr">
         <is>
           <t>Sparse cross-system presence (&lt; 7 sources)</t>
         </is>
       </c>
-      <c r="AI7" s="3" t="n">
+      <c r="AI7" s="4" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>GIS-0082</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>AI-Powered Contract Review &amp; Compliance Scanner</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>AI Team</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>Finance and Controls</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>Tualatin</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>Grace Lindqvist</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>Ingrid Iyer</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>Manager</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>Planning</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J8" s="3" t="inlineStr">
         <is>
           <t>2027-10-06</t>
         </is>
       </c>
-      <c r="K8" s="3" t="n">
+      <c r="K8" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="L8" s="3" t="n">
+      <c r="L8" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="M8" s="3" t="b">
+      <c r="M8" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="N8" s="3" t="b">
+      <c r="N8" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="O8" s="3" t="b">
+      <c r="O8" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="P8" s="2" t="inlineStr">
+      <c r="P8" s="3" t="inlineStr">
         <is>
           <t>Cybersecurity</t>
         </is>
       </c>
-      <c r="Q8" s="3" t="n">
+      <c r="Q8" s="4" t="n">
         <v>2.3</v>
       </c>
-      <c r="R8" s="3" t="n">
+      <c r="R8" s="4" t="n">
         <v>6500000</v>
       </c>
-      <c r="S8" s="3" t="n">
+      <c r="S8" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="T8" s="2" t="inlineStr">
+      <c r="T8" s="3" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="U8" s="3" t="n">
+      <c r="U8" s="4" t="n">
         <v>164</v>
       </c>
-      <c r="V8" s="3" t="n">
+      <c r="V8" s="4" t="n">
         <v>0.52</v>
       </c>
-      <c r="W8" s="3" t="n">
+      <c r="W8" s="4" t="n">
         <v>0.84</v>
       </c>
-      <c r="X8" s="3" t="n">
+      <c r="X8" s="4" t="n">
         <v>0.74</v>
       </c>
-      <c r="Y8" s="3" t="n">
+      <c r="Y8" s="4" t="n">
         <v>67.59999999999999</v>
       </c>
-      <c r="Z8" s="2" t="inlineStr">
+      <c r="Z8" s="3" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="AA8" s="2" t="inlineStr">
+      <c r="AA8" s="3" t="inlineStr">
         <is>
           <t>Can wait</t>
         </is>
       </c>
-      <c r="AB8" s="2" t="inlineStr">
+      <c r="AB8" s="3" t="inlineStr">
         <is>
           <t>Can wait</t>
         </is>
       </c>
-      <c r="AC8" s="3" t="n">
+      <c r="AC8" s="4" t="n">
         <v>52.9</v>
       </c>
-      <c r="AD8" s="2" t="inlineStr">
+      <c r="AD8" s="3" t="inlineStr">
         <is>
           <t>Re-sequence</t>
         </is>
       </c>
-      <c r="AE8" s="2" t="inlineStr">
+      <c r="AE8" s="3" t="inlineStr">
         <is>
           <t>Analytics</t>
         </is>
       </c>
-      <c r="AF8" s="2" t="inlineStr"/>
-      <c r="AG8" s="2" t="inlineStr">
+      <c r="AF8" s="3" t="inlineStr"/>
+      <c r="AG8" s="3" t="inlineStr">
         <is>
           <t>Business Value (+0.54); Timing Urgency (+0.30); Regulatory / Security (-0.12); Cost Magnitude (-0.33)</t>
         </is>
       </c>
-      <c r="AH8" s="2" t="inlineStr">
+      <c r="AH8" s="3" t="inlineStr">
         <is>
           <t>Sparse cross-system presence (&lt; 7 sources)</t>
         </is>
       </c>
-      <c r="AI8" s="3" t="n">
+      <c r="AI8" s="4" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>GIS-0083</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Autonomous Robotic Process AI Co-Pilot</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>AI Team</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>Manufacturing Engineering</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>Hsinchu</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>Owen Aziz</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>Nadia Novak</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>Executive</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I9" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J9" s="3" t="inlineStr">
         <is>
           <t>2027-04-13</t>
         </is>
       </c>
-      <c r="K9" s="3" t="n">
+      <c r="K9" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="L9" s="3" t="n">
+      <c r="L9" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="M9" s="3" t="b">
+      <c r="M9" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="N9" s="3" t="b">
+      <c r="N9" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="O9" s="3" t="b">
+      <c r="O9" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="P9" s="2" t="inlineStr">
+      <c r="P9" s="3" t="inlineStr">
         <is>
           <t>Unified Communications</t>
         </is>
       </c>
-      <c r="Q9" s="3" t="n">
+      <c r="Q9" s="4" t="n">
         <v>2.2</v>
       </c>
-      <c r="R9" s="3" t="n">
+      <c r="R9" s="4" t="n">
         <v>2170956</v>
       </c>
-      <c r="S9" s="3" t="n">
+      <c r="S9" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="T9" s="2" t="inlineStr">
+      <c r="T9" s="3" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="U9" s="3" t="n">
+      <c r="U9" s="4" t="n">
         <v>105</v>
       </c>
-      <c r="V9" s="3" t="n">
+      <c r="V9" s="4" t="n">
         <v>0.71</v>
       </c>
-      <c r="W9" s="3" t="n">
+      <c r="W9" s="4" t="n">
         <v>0.95</v>
       </c>
-      <c r="X9" s="3" t="n">
+      <c r="X9" s="4" t="n">
         <v>0.73</v>
       </c>
-      <c r="Y9" s="3" t="n">
+      <c r="Y9" s="4" t="n">
         <v>79.8</v>
       </c>
-      <c r="Z9" s="2" t="inlineStr">
+      <c r="Z9" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="AA9" s="2" t="inlineStr">
+      <c r="AA9" s="3" t="inlineStr">
         <is>
           <t>Proceed</t>
         </is>
       </c>
-      <c r="AB9" s="2" t="inlineStr">
+      <c r="AB9" s="3" t="inlineStr">
         <is>
           <t>Proceed</t>
         </is>
       </c>
-      <c r="AC9" s="3" t="n">
+      <c r="AC9" s="4" t="n">
         <v>74.90000000000001</v>
       </c>
-      <c r="AD9" s="2" t="inlineStr">
+      <c r="AD9" s="3" t="inlineStr">
         <is>
           <t>Proceed</t>
         </is>
       </c>
-      <c r="AE9" s="2" t="inlineStr">
+      <c r="AE9" s="3" t="inlineStr">
         <is>
           <t>Analytics</t>
         </is>
       </c>
-      <c r="AF9" s="2" t="inlineStr">
+      <c r="AF9" s="3" t="inlineStr">
         <is>
           <t>R2 Executive Sponsorship</t>
         </is>
       </c>
-      <c r="AG9" s="2" t="inlineStr">
+      <c r="AG9" s="3" t="inlineStr">
         <is>
           <t>Business Value (+0.72); Timing Urgency (+0.42); Regulatory / Security (-0.12); Cost Magnitude (-0.11)</t>
         </is>
       </c>
-      <c r="AH9" s="2" t="inlineStr"/>
-      <c r="AI9" s="3" t="n">
+      <c r="AH9" s="3" t="inlineStr"/>
+      <c r="AI9" s="4" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>GIS-0084</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Smart Energy Consumption Optimizer for Cleanrooms</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>AI Team</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>Global Supply Chain</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>Tualatin</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>Elena Rostova</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>Hannah Tanaka</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>Manager</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I10" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J10" s="3" t="inlineStr">
         <is>
           <t>2028-07-22</t>
         </is>
       </c>
-      <c r="K10" s="3" t="n">
+      <c r="K10" s="4" t="n">
         <v>30</v>
       </c>
-      <c r="L10" s="3" t="n">
+      <c r="L10" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="M10" s="3" t="b">
+      <c r="M10" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="N10" s="3" t="b">
+      <c r="N10" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="O10" s="3" t="b">
+      <c r="O10" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="P10" s="2" t="inlineStr">
+      <c r="P10" s="3" t="inlineStr">
         <is>
           <t>Cloud and Infrastructure</t>
         </is>
       </c>
-      <c r="Q10" s="3" t="n">
+      <c r="Q10" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="R10" s="3" t="n">
+      <c r="R10" s="4" t="n">
         <v>780000</v>
       </c>
-      <c r="S10" s="3" t="n">
+      <c r="S10" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="T10" s="2" t="inlineStr">
+      <c r="T10" s="3" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="U10" s="3" t="n">
+      <c r="U10" s="4" t="n">
         <v>72</v>
       </c>
-      <c r="V10" s="3" t="n">
+      <c r="V10" s="4" t="n">
         <v>0.72</v>
       </c>
-      <c r="W10" s="3" t="n">
+      <c r="W10" s="4" t="n">
         <v>0.83</v>
       </c>
-      <c r="X10" s="3" t="n">
+      <c r="X10" s="4" t="n">
         <v>0.82</v>
       </c>
-      <c r="Y10" s="3" t="n">
+      <c r="Y10" s="4" t="n">
         <v>77.90000000000001</v>
       </c>
-      <c r="Z10" s="2" t="inlineStr">
+      <c r="Z10" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="AA10" s="2" t="inlineStr">
+      <c r="AA10" s="3" t="inlineStr">
         <is>
           <t>Proceed</t>
         </is>
       </c>
-      <c r="AB10" s="2" t="inlineStr">
+      <c r="AB10" s="3" t="inlineStr">
         <is>
           <t>Must-do-now</t>
         </is>
       </c>
-      <c r="AC10" s="3" t="n">
+      <c r="AC10" s="4" t="n">
         <v>70</v>
       </c>
-      <c r="AD10" s="2" t="inlineStr">
+      <c r="AD10" s="3" t="inlineStr">
         <is>
           <t>Proceed</t>
         </is>
       </c>
-      <c r="AE10" s="2" t="inlineStr">
+      <c r="AE10" s="3" t="inlineStr">
         <is>
           <t>Core IT</t>
         </is>
       </c>
-      <c r="AF10" s="2" t="inlineStr">
+      <c r="AF10" s="3" t="inlineStr">
         <is>
           <t>R1 Regulatory First; R5 Cross-Portfolio Critical Path</t>
         </is>
       </c>
-      <c r="AG10" s="2" t="inlineStr">
+      <c r="AG10" s="3" t="inlineStr">
         <is>
           <t>Business Value (+0.36); Timing Urgency (+0.12); Regulatory / Security (+0.45); Cost Magnitude (-0.04)</t>
         </is>
       </c>
-      <c r="AH10" s="2" t="inlineStr">
+      <c r="AH10" s="3" t="inlineStr">
         <is>
           <t>High upstream dependency entanglement</t>
         </is>
       </c>
-      <c r="AI10" s="3" t="n">
+      <c r="AI10" s="4" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>GIS-0085</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>AI Model Safety, Guardrails &amp; Governance Suite</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>AI Team</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>Human Resources</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>Fremont</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>Yara Gallagher</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>Elena Ferreira</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H11" s="3" t="inlineStr">
         <is>
           <t>Executive</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I11" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="J11" s="3" t="inlineStr">
         <is>
           <t>2028-03-10</t>
         </is>
       </c>
-      <c r="K11" s="3" t="n">
+      <c r="K11" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="L11" s="3" t="n">
+      <c r="L11" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="M11" s="3" t="b">
+      <c r="M11" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="N11" s="3" t="b">
+      <c r="N11" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="O11" s="3" t="b">
+      <c r="O11" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="P11" s="2" t="inlineStr">
+      <c r="P11" s="3" t="inlineStr">
         <is>
           <t>Data Engineering</t>
         </is>
       </c>
-      <c r="Q11" s="3" t="n">
+      <c r="Q11" s="4" t="n">
         <v>8.4</v>
       </c>
-      <c r="R11" s="3" t="n">
+      <c r="R11" s="4" t="n">
         <v>610421</v>
       </c>
-      <c r="S11" s="3" t="n">
+      <c r="S11" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="T11" s="2" t="inlineStr">
+      <c r="T11" s="3" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="U11" s="3" t="n">
+      <c r="U11" s="4" t="n">
         <v>65</v>
       </c>
-      <c r="V11" s="3" t="n">
+      <c r="V11" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="W11" s="3" t="n">
+      <c r="W11" s="4" t="n">
         <v>0.89</v>
       </c>
-      <c r="X11" s="3" t="n">
+      <c r="X11" s="4" t="n">
         <v>0.72</v>
       </c>
-      <c r="Y11" s="3" t="n">
+      <c r="Y11" s="4" t="n">
         <v>90.59999999999999</v>
       </c>
-      <c r="Z11" s="2" t="inlineStr">
+      <c r="Z11" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="AA11" s="2" t="inlineStr">
+      <c r="AA11" s="3" t="inlineStr">
         <is>
           <t>Must-do-now</t>
         </is>
       </c>
-      <c r="AB11" s="2" t="inlineStr">
+      <c r="AB11" s="3" t="inlineStr">
         <is>
           <t>Must-do-now</t>
         </is>
       </c>
-      <c r="AC11" s="3" t="n">
+      <c r="AC11" s="4" t="n">
         <v>78.3</v>
       </c>
-      <c r="AD11" s="2" t="inlineStr">
+      <c r="AD11" s="3" t="inlineStr">
         <is>
           <t>Proceed</t>
         </is>
       </c>
-      <c r="AE11" s="2" t="inlineStr">
+      <c r="AE11" s="3" t="inlineStr">
         <is>
           <t>Analytics</t>
         </is>
       </c>
-      <c r="AF11" s="2" t="inlineStr">
+      <c r="AF11" s="3" t="inlineStr">
         <is>
           <t>R1 Regulatory First</t>
         </is>
       </c>
-      <c r="AG11" s="2" t="inlineStr">
+      <c r="AG11" s="3" t="inlineStr">
         <is>
           <t>Business Value (+0.54); Timing Urgency (+0.20); Regulatory / Security (+0.45); Cost Magnitude (-0.03)</t>
         </is>
       </c>
-      <c r="AH11" s="2" t="inlineStr"/>
-      <c r="AI11" s="3" t="n">
+      <c r="AH11" s="3" t="inlineStr"/>
+      <c r="AI11" s="4" t="n">
         <v>11</v>
       </c>
     </row>

</xml_diff>